<commit_message>
update v15 com UI novas e refatoraracao e modelagem com notebooks para o artigo cientico
</commit_message>
<xml_diff>
--- a/lib/hash_table.xlsx
+++ b/lib/hash_table.xlsx
@@ -437,1082 +437,1082 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>15.54531838293458</v>
+        <v>26.05845476919577</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>14.66410218309929</v>
+        <v>22.86600961511795</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>12.44995122914631</v>
+        <v>21.64736113255699</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>7.778152495954682</v>
+        <v>18.6144625992209</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>7.378868840111652</v>
+        <v>17.36819739724094</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>6.700222752642359</v>
+        <v>17.02360507988341</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>6.679901416981371</v>
+        <v>16.55407615166203</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>6.232889988004143</v>
+        <v>15.77900665531947</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>6.078610417987518</v>
+        <v>15.54531838293443</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>5.601896270963724</v>
+        <v>14.66410218309929</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>5.245654095095698</v>
+        <v>13.3447267903799</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>5.230808144247745</v>
+        <v>12.44995122914663</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>5.104770821357429</v>
+        <v>10.65512917904204</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>5.104767181518222</v>
+        <v>8.913627025534243</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>5.0586650418178</v>
+        <v>8.335508550897774</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>5.036408924477143</v>
+        <v>8.275535183571348</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>5.021573723728667</v>
+        <v>8.240447025363707</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>4.916023145354487</v>
+        <v>7.908005312866873</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>4.904649436675812</v>
+        <v>7.788605641411117</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>4.831524459184733</v>
+        <v>7.665195775008982</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>4.813943547329425</v>
+        <v>7.542073792847603</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>4.736889059669469</v>
+        <v>7.378868840111763</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>4.726224018944181</v>
+        <v>7.024423915842871</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>4.722595506367155</v>
+        <v>6.73650542439198</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>4.71218879506925</v>
+        <v>6.679901416981259</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>4.71218562740654</v>
+        <v>6.633690869228259</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>4.707771730101995</v>
+        <v>6.338943322872359</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>4.604259769292107</v>
+        <v>6.297195687874957</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>4.49506888472706</v>
+        <v>6.232889988004087</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>4.452265614177953</v>
+        <v>6.078610417987607</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>4.449494715575342</v>
+        <v>6.073739126008116</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>4.446725358595827</v>
+        <v>5.601896270963658</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>4.432364585717341</v>
+        <v>5.288815940683255</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>4.418143663341567</v>
+        <v>5.245654095095698</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>4.404089826112267</v>
+        <v>5.230808144247701</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>4.38829151753326</v>
+        <v>5.104770821357563</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>4.388291517533238</v>
+        <v>5.104767181518222</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>4.388291517533216</v>
+        <v>5.0586650418176</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>4.388291517533216</v>
+        <v>5.041536772765931</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>4.388291517533216</v>
+        <v>5.03640892447712</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>4.388291517533216</v>
+        <v>5.021573723728667</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>4.388291517533194</v>
+        <v>4.924888436226138</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>4.388291517533194</v>
+        <v>4.91891351310707</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>4.388291517533172</v>
+        <v>4.916023145354398</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>4.388291517533172</v>
+        <v>4.916017807544404</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>4.388291517533149</v>
+        <v>4.904649436675812</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>4.388291517533127</v>
+        <v>4.888685947150639</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>4.388291517533127</v>
+        <v>4.831524459184755</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>4.388291517533083</v>
+        <v>4.814396056529979</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>4.349633931007113</v>
+        <v>4.813943547329447</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>4.349633931007069</v>
+        <v>4.736889059669314</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>4.34963393100698</v>
+        <v>4.726224018944181</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>4.325966886632271</v>
+        <v>4.722595506367155</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>4.274519009916911</v>
+        <v>4.71218879506925</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>4.270257231299013</v>
+        <v>4.712185627406562</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>4.23344250423825</v>
+        <v>4.70926335620534</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>4.233442504238227</v>
+        <v>4.707771730101995</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>4.233442504238205</v>
+        <v>4.687572527072725</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
-        <v>4.233442504238205</v>
+        <v>4.685691472398901</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
-        <v>4.233442504238183</v>
+        <v>4.669201329720174</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
-        <v>4.233442504238183</v>
+        <v>4.604261815148591</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
-        <v>4.233442504238183</v>
+        <v>4.604259769292196</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
-        <v>4.233442504238161</v>
+        <v>4.49506888472706</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>4.219071160432186</v>
+        <v>4.475571792297295</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
-        <v>4.19406792021233</v>
+        <v>4.46061635483932</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
-        <v>4.175848843858931</v>
+        <v>4.452269003190468</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
-        <v>4.168259217128245</v>
+        <v>4.452265614177953</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>4.16099973736932</v>
+        <v>4.449494715575342</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>4.152707281016244</v>
+        <v>4.44672724950923</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>4.139113523896243</v>
+        <v>4.446725358595827</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>4.000000000000048</v>
+        <v>4.418143663341567</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
-        <v>4.000000000000048</v>
+        <v>4.404089826112356</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
-        <v>4.000000000000048</v>
+        <v>4.388291517533238</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>4.000000000000026</v>
+        <v>4.388291517533238</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
-        <v>4.000000000000026</v>
+        <v>4.388291517533216</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
-        <v>4.000000000000026</v>
+        <v>4.388291517533216</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
-        <v>4.000000000000026</v>
+        <v>4.388291517533216</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>4.000000000000026</v>
+        <v>4.388291517533216</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
-        <v>4.000000000000026</v>
+        <v>4.388291517533194</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
-        <v>4.000000000000004</v>
+        <v>4.388291517533172</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
-        <v>4.000000000000004</v>
+        <v>4.388291517533172</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
-        <v>4.000000000000004</v>
+        <v>4.388291517533172</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>4.000000000000004</v>
+        <v>4.388291517533172</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>4.000000000000004</v>
+        <v>4.388291517533172</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
-        <v>4.000000000000004</v>
+        <v>4.388291517533172</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>4.000000000000004</v>
+        <v>4.388291517533149</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
-        <v>4.000000000000004</v>
+        <v>4.388291517533127</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
-        <v>3.999999999999981</v>
+        <v>4.388291517533127</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>3.999999999999981</v>
+        <v>4.349633931007113</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
-        <v>3.999999999999981</v>
+        <v>4.349633931007091</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>3.999999999999981</v>
+        <v>4.349633931007069</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
-        <v>3.999999999999981</v>
+        <v>4.349633931007046</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>3.999999999999981</v>
+        <v>4.349633931007046</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
-        <v>3.999999999999981</v>
+        <v>4.349633931007046</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>3.999999999999981</v>
+        <v>4.349633931007046</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
-        <v>3.999999999999981</v>
+        <v>4.349633931007046</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
-        <v>3.999999999999981</v>
+        <v>4.349633931007046</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>3.999999999999981</v>
+        <v>4.349633931007024</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
-        <v>3.999999999999959</v>
+        <v>4.349633931007024</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
-        <v>3.999999999999959</v>
+        <v>4.349633931007002</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>3.999999999999959</v>
+        <v>4.34963393100698</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
-        <v>3.999999999999937</v>
+        <v>4.34963393100698</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
-        <v>3.999999999999937</v>
+        <v>4.34963393100698</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>3.999999999999937</v>
+        <v>4.335477316788561</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
-        <v>3.999999999999937</v>
+        <v>4.335475298823388</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
-        <v>-1</v>
+        <v>4.325966886632249</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>-1</v>
+        <v>4.274519009916911</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
-        <v>-1</v>
+        <v>4.270257231299013</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
-        <v>-1</v>
+        <v>4.23344250423825</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
-        <v>-1</v>
+        <v>4.23344250423825</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
-        <v>-1</v>
+        <v>4.23344250423825</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
-        <v>-1</v>
+        <v>4.23344250423825</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
-        <v>-1</v>
+        <v>4.233442504238227</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
-        <v>-1</v>
+        <v>4.233442504238227</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
-        <v>-1</v>
+        <v>4.233442504238227</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
-        <v>-1</v>
+        <v>4.233442504238227</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
-        <v>-1</v>
+        <v>4.233442504238227</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
-        <v>-1</v>
+        <v>4.233442504238227</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
-        <v>-1</v>
+        <v>4.233442504238227</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
-        <v>-1</v>
+        <v>4.233442504238205</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
-        <v>-1</v>
+        <v>4.233442504238205</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
-        <v>-1</v>
+        <v>4.233442504238205</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
-        <v>-1</v>
+        <v>4.233442504238205</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
-        <v>-1</v>
+        <v>4.233442504238205</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
-        <v>-1</v>
+        <v>4.233442504238205</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
-        <v>-1</v>
+        <v>4.233442504238183</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
-        <v>-1</v>
+        <v>4.233442504238183</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
-        <v>-1</v>
+        <v>4.233442504238183</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
-        <v>-1</v>
+        <v>4.233442504238183</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
-        <v>-1</v>
+        <v>4.233442504238183</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
-        <v>-1</v>
+        <v>4.233442504238183</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
-        <v>-1</v>
+        <v>4.233442504238183</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
-        <v>-1</v>
+        <v>4.233442504238161</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
-        <v>-1</v>
+        <v>4.233442504238161</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
-        <v>-1</v>
+        <v>4.233442504238161</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
-        <v>-1</v>
+        <v>4.233442504238139</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
-        <v>-1</v>
+        <v>4.233442504238139</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
-        <v>-1</v>
+        <v>4.233442504238139</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
-        <v>-1</v>
+        <v>4.233442504238139</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
-        <v>-1</v>
+        <v>4.233442504238139</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
-        <v>-1</v>
+        <v>4.233442504238116</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
-        <v>-1</v>
+        <v>4.233442504238116</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
-        <v>-1</v>
+        <v>4.233442504238094</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
-        <v>-1</v>
+        <v>4.219071160432186</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
-        <v>-1</v>
+        <v>4.194067920212374</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
-        <v>-1</v>
+        <v>4.175848843858931</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
-        <v>-1</v>
+        <v>4.169529680102513</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
-        <v>-1</v>
+        <v>4.168261095111214</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
-        <v>-1</v>
+        <v>4.168259217128245</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
-        <v>-1</v>
+        <v>4.16099973736932</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
-        <v>-1</v>
+        <v>4.152707281016221</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
-        <v>-1</v>
+        <v>4.139113523896243</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
-        <v>-1</v>
+        <v>4.11804620363041</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
-        <v>-1</v>
+        <v>4.061116337551218</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
-        <v>-1</v>
+        <v>4.00797224759124</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
-        <v>-1</v>
+        <v>4.000000000000048</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
-        <v>-1</v>
+        <v>4.000000000000048</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
-        <v>-1</v>
+        <v>4.000000000000048</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
-        <v>-1</v>
+        <v>4.000000000000048</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
-        <v>-1</v>
+        <v>4.000000000000026</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
-        <v>-1</v>
+        <v>4.000000000000026</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
-        <v>-1</v>
+        <v>4.000000000000026</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
-        <v>-1</v>
+        <v>4.000000000000026</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
-        <v>-1</v>
+        <v>4.000000000000026</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
-        <v>-1</v>
+        <v>4.000000000000026</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
-        <v>-1</v>
+        <v>4.000000000000026</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
-        <v>-1</v>
+        <v>4.000000000000026</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
-        <v>-1</v>
+        <v>4.000000000000026</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
-        <v>-1</v>
+        <v>4.000000000000026</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
-        <v>-1</v>
+        <v>4.000000000000026</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
-        <v>-1</v>
+        <v>4.000000000000026</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
-        <v>-1</v>
+        <v>4.000000000000026</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
-        <v>-1</v>
+        <v>4.000000000000004</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
-        <v>-1</v>
+        <v>3.999999999999981</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
-        <v>-1</v>
+        <v>3.999999999999981</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
-        <v>-1</v>
+        <v>3.999999999999981</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
-        <v>-1</v>
+        <v>3.999999999999981</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
-        <v>-1</v>
+        <v>3.999999999999981</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
-        <v>-1</v>
+        <v>3.999999999999981</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
-        <v>-1</v>
+        <v>3.999999999999981</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
-        <v>-1</v>
+        <v>3.999999999999981</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
-        <v>-1</v>
+        <v>3.999999999999981</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="n">
-        <v>-1</v>
+        <v>3.999999999999981</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="n">
-        <v>-1</v>
+        <v>3.999999999999981</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="n">
-        <v>-1</v>
+        <v>3.999999999999981</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="n">
-        <v>-1</v>
+        <v>3.999999999999981</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="n">
-        <v>-1</v>
+        <v>3.999999999999959</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="n">
-        <v>-1</v>
+        <v>3.999999999999959</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="n">
-        <v>-1</v>
+        <v>3.999999999999959</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="n">
-        <v>-1</v>
+        <v>3.999999999999959</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
-        <v>-1</v>
+        <v>3.999999999999959</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="n">
-        <v>-1</v>
+        <v>3.999999999999959</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
-        <v>-1</v>
+        <v>3.999999999999959</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="n">
-        <v>-1</v>
+        <v>3.999999999999937</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
-        <v>-1</v>
+        <v>3.999999999999937</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
-        <v>-1</v>
+        <v>3.999999999999937</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="n">
-        <v>-1</v>
+        <v>3.999999999999937</v>
       </c>
     </row>
     <row r="218">

</xml_diff>